<commit_message>
feat(planos): reduz minimo mensal dos pacotes, remove chip Livre e atualiza cronograma mobile
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TABELA_PRECOS_ZELA.xlsx
+++ b/docs/TABELA_PRECOS_ZELA.xlsx
@@ -737,13 +737,13 @@
       <c r="B13" s="9" t="n"/>
       <c r="C13" s="9" t="n"/>
       <c r="D13" s="11" t="n">
-        <v>450</v>
+        <v>290</v>
       </c>
       <c r="E13" s="11" t="n">
-        <v>790</v>
+        <v>490</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>990</v>
+        <v>690</v>
       </c>
     </row>
     <row r="14">
@@ -764,6 +764,7 @@
         <v>1908</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>

</xml_diff>